<commit_message>
workbook: add FoldX monomer ddG column + BRCT sheet with threshold sweep
- Benchmark_per_variant: foldx_ddg_monomer[/_sd/_confident] for all 44 variants
- New sheet Benchmark_BRCT_foldx: 12 BRCT variants vs measured GdmCl unfolding ddG
  (Rowling 2010, JBC 285:20080), fold-axis token agreement 10/12 stable across
  t=1.0/1.5/2.0/2.5 and Sapozhnikov per-axis (mono=2.9); legacy t=2.5 classification
  column (9/12) retained and relabeled
- README_corrections: 2 provenance rows
</commit_message>
<xml_diff>
--- a/reference_outputs/MAVIS_results_summary.xlsx
+++ b/reference_outputs/MAVIS_results_summary.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_corrections" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark_per_variant" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark_tier_calibration" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark_AM_accuracy" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark_AM_error_cases" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark_mechanism_dist" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHD_per_variant" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHD_control_recall_3thr" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHD_concordance_dist_3thr" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHD_candidates_3thr" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHD_orthogonal_cases" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="README_corrections" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Benchmark_per_variant" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Benchmark_tier_calibration" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Benchmark_AM_accuracy" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Benchmark_AM_error_cases" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Benchmark_mechanism_dist" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CHD_per_variant" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CHD_control_recall_3thr" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="CHD_concordance_dist_3thr" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="CHD_candidates_3thr" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="CHD_orthogonal_cases" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Benchmark_BRCT_foldx" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47,7 +48,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -55,14 +56,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -429,20 +439,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>detail</t>
         </is>
@@ -613,6 +619,30 @@
       <c r="B15" t="inlineStr">
         <is>
           <t>Pearson 0.570 / Spearman 0.468 (tier-strength vs AM, 44 variants)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>FoldX monomer ddG (v6)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Benchmark_per_variant: foldx_ddg_monomer[/_sd/_confident] added for all 44 variants (FoldX 5.1 BuildModel n=5, kcal/mol).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BRCT monomer-fold arm (v6)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>New sheet Benchmark_BRCT_foldx: 12 BRCA1 BRCT variants vs measured GdmCl unfolding ddG (Rowling 2010, JBC 285:20080). Fold-axis agreement 9/12 @ t=2.5.</t>
         </is>
       </c>
     </row>
@@ -1519,86 +1549,1086 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>variant</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>truth_role</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>clinvar_germline</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>role_in_cohort</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>site_class</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>measured_ddG_U-F_kcal_mol</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>foldx_ddg_monomer</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>foldx_ddg_sd</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>rowling2010_reported_foldx_ddG</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>measured_destab</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>foldx_call_destab</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>agreement_t2.5_classification_legacy</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>agree_t1.0</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>agree_t1.5</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>agree_t2.0</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>agree_t2.5</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>agree_t_Sapozhnikov_mono2.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Y1853C</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>pathogenic</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Pathogenic/Likely pathogenic</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>monomer_fold_destabilizer</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>core/fold</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3.3869</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.1766</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>A1843P</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pathogenic</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Likely pathogenic</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>monomer_fold_destabilizer</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>core/fold</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6.4287</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="I3" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>V1736A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pathogenic</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Pathogenic</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>monomer_fold_destabilizer</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>core/fold</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.2414</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J4" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>M1783T</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>conflicting</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Conflicting classifications of pathogenicity</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>monomer_fold_destabilizer</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>core/fold</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2.8551</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.06560000000000001</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>V1808A</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>vus</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Uncertain significance</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>monomer_fold_destabilizer</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>core/fold</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3.5669</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.0258</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>V1665M</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>conflicting</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Conflicting classifications of pathogenicity</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>monomer_fold_destabilizer</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>core/fold</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2.979</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.3602</v>
+      </c>
+      <c r="I7" t="n">
+        <v>8.59</v>
+      </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>R1751Q</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>benign</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>monomer_fold_destabilizer</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>core/fold</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.7285</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.07829999999999999</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K8" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>L1664P</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>benign</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Benign</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>monomer_fold_destabilizer</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>core/fold</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.5333</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.07439999999999999</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>M1663K</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>vus</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Uncertain significance</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>measured_neutral_control</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>core/fold</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.4458</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.0449</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K10" t="b">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>P1806A</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>conflicting</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Conflicting classifications of pathogenicity</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>measured_neutral_control</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>core/fold</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.6691</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11" t="b">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>R1699L</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>pathogenic</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Likely pathogenic</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>fold_intact_function_lost</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>binding_groove/surface</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>-0.99</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.387</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.5647</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="J12" t="b">
+        <v>0</v>
+      </c>
+      <c r="K12" t="b">
+        <v>0</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>R1699Q</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>pathogenic</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Pathogenic</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>fold_intact_function_lost</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>binding_groove/surface</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>-1.83</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.768</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J13" t="b">
+        <v>0</v>
+      </c>
+      <c r="K13" t="b">
+        <v>0</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>DISAGREE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>gene</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>variant</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>truth_role</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>mavis_structural_evidence</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>mavis_mechanism</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>foldx_ddg_monomer</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>foldx_ddg_monomer_sd</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>foldx_monomer_confident</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>axis_corrob_monomer</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>axis_corrob_fold</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>axis_corrob_binding</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>AM_score</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>AM_class</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>AM_vs_truth</t>
         </is>
@@ -1635,30 +2665,39 @@
           <t>Both fold + PPI destabilization</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="n">
+        <v>1.4503</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>corroborated_disruption</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>corroborated_disruption</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="M2" t="n">
         <v>0.705</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -1695,30 +2734,39 @@
           <t>Both fold destabilization</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="n">
+        <v>2.3282</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.0456</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="M3" t="n">
         <v>0.99</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -1755,30 +2803,39 @@
           <t>No structural effect detected</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="n">
+        <v>0.1193</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.0263</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="M4" t="n">
         <v>0.081</v>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>likely_benign</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -1815,30 +2872,39 @@
           <t>No structural effect detected</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="n">
+        <v>-0.3113</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.0267</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="M5" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>likely_benign</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -1875,30 +2941,39 @@
           <t>Multimer fold destabilization at interface</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="n">
+        <v>0.0062</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="M6" t="n">
         <v>0.9409999999999999</v>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -1935,30 +3010,39 @@
           <t>Multimer fold destab. + PPI stabilization (conflicting)</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.0342</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="M7" t="n">
         <v>0.988</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -1995,30 +3079,39 @@
           <t>Multimer fold destabilization</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" t="n">
+        <v>-1.5867</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.5009</v>
+      </c>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="M8" t="n">
         <v>0.538</v>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>ambiguous</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>ambiguous</t>
         </is>
@@ -2055,30 +3148,39 @@
           <t>Both fold + PPI destabilization</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" t="n">
+        <v>2.1325</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.5089</v>
+      </c>
+      <c r="I9" t="b">
+        <v>1</v>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J9" t="n">
+      <c r="M9" t="n">
         <v>0.999</v>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2115,30 +3217,39 @@
           <t>No structural effect detected</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" t="n">
+        <v>0.4337</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.0446</v>
+      </c>
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J10" t="n">
+      <c r="M10" t="n">
         <v>0.253</v>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>likely_benign</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2175,30 +3286,39 @@
           <t>Multimer fold destabilization at interface</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" t="n">
+        <v>-0.7965</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.0351</v>
+      </c>
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>corroborated_disruption</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J11" t="n">
+      <c r="M11" t="n">
         <v>0.918</v>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2235,30 +3355,39 @@
           <t>Multimer fold + PPI destabilization</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" t="n">
+        <v>0.9510999999999999</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.0842</v>
+      </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J12" t="n">
+      <c r="M12" t="n">
         <v>0.999</v>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2295,30 +3424,39 @@
           <t>PPI stabilization</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" t="n">
+        <v>0.9673</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.1677</v>
+      </c>
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J13" t="n">
+      <c r="M13" t="n">
         <v>0.986</v>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2355,30 +3493,39 @@
           <t>Multimer fold destab. + PPI stabilization (conflicting)</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" t="n">
+        <v>-0.8679</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.0353</v>
+      </c>
+      <c r="I14" t="b">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J14" t="n">
+      <c r="M14" t="n">
         <v>0.988</v>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>FP</t>
         </is>
@@ -2415,30 +3562,39 @@
           <t>Interface variant (DDG neutral)</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" t="n">
+        <v>-0.8024</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="I15" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J15" t="n">
+      <c r="M15" t="n">
         <v>0.077</v>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>likely_benign</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2475,30 +3631,39 @@
           <t>Multimer fold stabilization</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.0125</v>
+      </c>
+      <c r="I16" t="b">
+        <v>1</v>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J16" t="n">
+      <c r="M16" t="n">
         <v>0.225</v>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>likely_benign</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2535,30 +3700,39 @@
           <t>Both fold destabilization</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" t="n">
+        <v>1.0894</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.0151</v>
+      </c>
+      <c r="I17" t="b">
+        <v>1</v>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J17" t="n">
+      <c r="M17" t="n">
         <v>0.649</v>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>FP</t>
         </is>
@@ -2595,30 +3769,39 @@
           <t>Both fold destabilization</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" t="n">
+        <v>3.9881</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.5288</v>
+      </c>
+      <c r="I18" t="b">
+        <v>1</v>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>corroborated_disruption_redundant</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J18" t="n">
+      <c r="M18" t="n">
         <v>0.999</v>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2655,30 +3838,39 @@
           <t>Both fold destabilization</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" t="n">
+        <v>4.8866</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.1741</v>
+      </c>
+      <c r="I19" t="b">
+        <v>1</v>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J19" t="n">
+      <c r="M19" t="n">
         <v>0.896</v>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2715,30 +3907,39 @@
           <t>Both fold destabilization</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" t="n">
+        <v>13.2941</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.2767</v>
+      </c>
+      <c r="I20" t="b">
+        <v>1</v>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>corroborated_disruption_redundant</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J20" t="n">
+      <c r="M20" t="n">
         <v>0.991</v>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2775,30 +3976,39 @@
           <t>Monomer fold destabilization</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" t="n">
+        <v>1.4817</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.0567</v>
+      </c>
+      <c r="I21" t="b">
+        <v>1</v>
+      </c>
+      <c r="J21" t="inlineStr">
         <is>
           <t>corroborated_disruption_redundant</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J21" t="n">
+      <c r="M21" t="n">
         <v>0.348</v>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>ambiguous</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>ambiguous</t>
         </is>
@@ -2835,30 +4045,39 @@
           <t>Multimer fold destabilization</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" t="n">
+        <v>-0.09130000000000001</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.0447</v>
+      </c>
+      <c r="I22" t="b">
+        <v>0</v>
+      </c>
+      <c r="J22" t="inlineStr">
         <is>
           <t>corroborated_silent</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J22" t="n">
+      <c r="M22" t="n">
         <v>0.323</v>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>likely_benign</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2895,30 +4114,39 @@
           <t>Multimer fold + PPI destabilization</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" t="n">
+        <v>-0.1901</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.0372</v>
+      </c>
+      <c r="I23" t="b">
+        <v>1</v>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J23" t="n">
+      <c r="M23" t="n">
         <v>0.996</v>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -2955,30 +4183,39 @@
           <t>Both fold destabilization</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" t="n">
+        <v>4.1145</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.3748</v>
+      </c>
+      <c r="I24" t="b">
+        <v>1</v>
+      </c>
+      <c r="J24" t="inlineStr">
         <is>
           <t>corroborated_disruption_redundant</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="J24" t="n">
+      <c r="M24" t="n">
         <v>0.999</v>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3015,30 +4252,39 @@
           <t>Both fold destabilization</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" t="n">
+        <v>1.285</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.0379</v>
+      </c>
+      <c r="I25" t="b">
+        <v>1</v>
+      </c>
+      <c r="J25" t="inlineStr">
         <is>
           <t>corroborated_disruption_redundant</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J25" t="n">
+      <c r="M25" t="n">
         <v>0.973</v>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3075,30 +4321,39 @@
           <t>Multimer fold stabilization</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" t="n">
+        <v>-0.1249</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.0122</v>
+      </c>
+      <c r="I26" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>corroborated_silent</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J26" t="n">
+      <c r="M26" t="n">
         <v>0.998</v>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3135,30 +4390,39 @@
           <t>No structural effect detected</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" t="n">
+        <v>0.4266</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.0687</v>
+      </c>
+      <c r="I27" t="b">
+        <v>1</v>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>corroborated_silent</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J27" t="n">
+      <c r="M27" t="n">
         <v>0.995</v>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3195,30 +4459,39 @@
           <t>No structural effect detected</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" t="n">
+        <v>0.7045</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.0218</v>
+      </c>
+      <c r="I28" t="b">
+        <v>1</v>
+      </c>
+      <c r="J28" t="inlineStr">
         <is>
           <t>corroborated_silent</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J28" t="n">
+      <c r="M28" t="n">
         <v>0.998</v>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3255,30 +4528,39 @@
           <t>No structural effect detected</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" t="n">
+        <v>0.717</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.1257</v>
+      </c>
+      <c r="I29" t="b">
+        <v>1</v>
+      </c>
+      <c r="J29" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J29" t="n">
+      <c r="M29" t="n">
         <v>0.223</v>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>likely_benign</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>FN</t>
         </is>
@@ -3315,30 +4597,39 @@
           <t>Multimer fold + PPI destabilization</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" t="n">
+        <v>0.2176</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.0231</v>
+      </c>
+      <c r="I30" t="b">
+        <v>1</v>
+      </c>
+      <c r="J30" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J30" t="n">
+      <c r="M30" t="n">
         <v>0.894</v>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3375,30 +4666,39 @@
           <t>Both fold + PPI destabilization</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" t="n">
+        <v>1.8174</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="I31" t="b">
+        <v>1</v>
+      </c>
+      <c r="J31" t="inlineStr">
         <is>
           <t>corroborated_disruption</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J31" t="n">
+      <c r="M31" t="n">
         <v>0.969</v>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3435,30 +4735,39 @@
           <t>Both fold + PPI destabilization</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" t="n">
+        <v>2.4086</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.0269</v>
+      </c>
+      <c r="I32" t="b">
+        <v>1</v>
+      </c>
+      <c r="J32" t="inlineStr">
         <is>
           <t>corroborated_disruption</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J32" t="n">
+      <c r="M32" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3495,30 +4804,39 @@
           <t>Multimer fold + PPI destabilization</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" t="n">
+        <v>0.6781</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="I33" t="b">
+        <v>1</v>
+      </c>
+      <c r="J33" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J33" t="n">
+      <c r="M33" t="n">
         <v>0.993</v>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3555,30 +4873,39 @@
           <t>Interface variant (DDG neutral)</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" t="n">
+        <v>-0.7689</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.07969999999999999</v>
+      </c>
+      <c r="I34" t="b">
+        <v>1</v>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J34" t="n">
+      <c r="M34" t="n">
         <v>0.969</v>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3615,30 +4942,39 @@
           <t>Both fold destabilization at interface</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" t="n">
+        <v>2.0291</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.0233</v>
+      </c>
+      <c r="I35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J35" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J35" t="n">
+      <c r="M35" t="n">
         <v>0.971</v>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3675,30 +5011,39 @@
           <t>Multimer fold destabilization at interface</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.0343</v>
+      </c>
+      <c r="I36" t="b">
+        <v>1</v>
+      </c>
+      <c r="J36" t="inlineStr">
         <is>
           <t>corroborated_silent</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J36" t="n">
+      <c r="M36" t="n">
         <v>0.6870000000000001</v>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="O36" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3735,30 +5080,39 @@
           <t>Multimer fold destabilization at interface</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G37" t="n">
+        <v>0.9203</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.0669</v>
+      </c>
+      <c r="I37" t="b">
+        <v>1</v>
+      </c>
+      <c r="J37" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>corroborated_disruption</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="J37" t="n">
+      <c r="M37" t="n">
         <v>0.411</v>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>ambiguous</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>ambiguous</t>
         </is>
@@ -3795,30 +5149,39 @@
           <t>No structural effect detected</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G38" t="n">
+        <v>0.6571</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.0166</v>
+      </c>
+      <c r="I38" t="b">
+        <v>1</v>
+      </c>
+      <c r="J38" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J38" t="n">
+      <c r="M38" t="n">
         <v>0.127</v>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>likely_benign</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3855,30 +5218,39 @@
           <t>PPI stabilization</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G39" t="n">
+        <v>0.4139</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.5286</v>
+      </c>
+      <c r="I39" t="b">
+        <v>1</v>
+      </c>
+      <c r="J39" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J39" t="n">
+      <c r="M39" t="n">
         <v>0.984</v>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="O39" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -3915,30 +5287,39 @@
           <t>No structural effect detected</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.0173</v>
+      </c>
+      <c r="I40" t="b">
+        <v>1</v>
+      </c>
+      <c r="J40" t="inlineStr">
         <is>
           <t>corroborated_silent</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J40" t="n">
+      <c r="M40" t="n">
         <v>0.209</v>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>likely_benign</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>FN</t>
         </is>
@@ -3975,30 +5356,39 @@
           <t>Interface variant (DDG neutral)</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" t="n">
+        <v>0.706</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="I41" t="b">
+        <v>1</v>
+      </c>
+      <c r="J41" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>channels_conflict</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J41" t="n">
+      <c r="M41" t="n">
         <v>0.998</v>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="O41" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -4035,30 +5425,39 @@
           <t>Both fold destabilization</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G42" t="n">
+        <v>12.1121</v>
+      </c>
+      <c r="H42" t="n">
+        <v>3.4371</v>
+      </c>
+      <c r="I42" t="b">
+        <v>1</v>
+      </c>
+      <c r="J42" t="inlineStr">
         <is>
           <t>corroborated_disruption_redundant</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J42" t="n">
-        <v>1</v>
-      </c>
-      <c r="K42" t="inlineStr">
+      <c r="M42" t="n">
+        <v>1</v>
+      </c>
+      <c r="N42" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="O42" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -4095,30 +5494,39 @@
           <t>Both fold + PPI destabilization</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G43" t="n">
+        <v>2.7454</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.2665</v>
+      </c>
+      <c r="I43" t="b">
+        <v>1</v>
+      </c>
+      <c r="J43" t="inlineStr">
         <is>
           <t>corroborated_disruption</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>corroborated_disruption</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J43" t="n">
+      <c r="M43" t="n">
         <v>0.998</v>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="O43" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -4155,30 +5563,39 @@
           <t>Monomer fold destabilization</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" t="n">
+        <v>1.6233</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="I44" t="b">
+        <v>1</v>
+      </c>
+      <c r="J44" t="inlineStr">
         <is>
           <t>corroborated_disruption_redundant</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J44" t="n">
+      <c r="M44" t="n">
         <v>0.991</v>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="N44" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="O44" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -4215,30 +5632,39 @@
           <t>No structural effect detected</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" t="n">
+        <v>0.9476</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="I45" t="b">
+        <v>1</v>
+      </c>
+      <c r="J45" t="inlineStr">
         <is>
           <t>corroborated_silent</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>ddg_unevaluable</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>has_ground_truth</t>
         </is>
       </c>
-      <c r="J45" t="n">
+      <c r="M45" t="n">
         <v>0.616</v>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="N45" t="inlineStr">
         <is>
           <t>likely_pathogenic</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="O45" t="inlineStr">
         <is>
           <t>correct</t>
         </is>

</xml_diff>